<commit_message>
ADO parser updated to also create feature->stories hierarchy from the uploaded export having multiple features
</commit_message>
<xml_diff>
--- a/ado-extract-partial-novation-phase1.xlsx
+++ b/ado-extract-partial-novation-phase1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chetan\ai-learning-lab\knowledge-drift-detector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8520284-E09C-4F98-A563-67E79E8B3405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA18D82-C5AB-4186-8FF3-3469D47C7228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{EB8649F9-5116-47FC-AF09-DC24D508B048}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="44">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -174,6 +174,13 @@
   </si>
   <si>
     <t>State</t>
+  </si>
+  <si>
+    <t>Combine Full and partial novation in one action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On the action menu user sees only one action called novation. Upon taking this action, when the trade launches in novation mode then user can select between Full or Partial novation. That selection to drive the behavior of the event
+</t>
   </si>
 </sst>
 </file>
@@ -539,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C538EE90-A18A-4E80-BFE3-D4A0E37F34E7}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.08984375" bestFit="1" customWidth="1"/>
@@ -842,6 +849,27 @@
         <v>34</v>
       </c>
     </row>
+    <row r="14" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>21223</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="2">
+        <v>23356</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added feature resolution & selection logic based in keyword match and fuzzy logic
</commit_message>
<xml_diff>
--- a/ado-extract-partial-novation-phase1.xlsx
+++ b/ado-extract-partial-novation-phase1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chetan\ai-learning-lab\knowledge-drift-detector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA18D82-C5AB-4186-8FF3-3469D47C7228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DFD818-12D0-49D4-9FF8-904D58F86077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{EB8649F9-5116-47FC-AF09-DC24D508B048}"/>
   </bookViews>
@@ -54,14 +54,8 @@
     <t>subtask</t>
   </si>
   <si>
-    <t>Partail Novation phase 1</t>
-  </si>
-  <si>
     <t>Supporting manual partial novation. User can take a new action partial novation on a trade and input novation details like new counterparty, novation date time, event reason etc and submit the event. 
 New trade creation against the new cpty has to be done manually as a fresh trade booking</t>
-  </si>
-  <si>
-    <t>Partial Novation Phase 2</t>
   </si>
   <si>
     <t>Automated trade creation against the new cpty from the original trade when partial novation event is performed on an existing trade</t>
@@ -181,6 +175,12 @@
   <si>
     <t xml:space="preserve">On the action menu user sees only one action called novation. Upon taking this action, when the trade launches in novation mode then user can select between Full or Partial novation. That selection to drive the behavior of the event
 </t>
+  </si>
+  <si>
+    <t>Partial Termination</t>
+  </si>
+  <si>
+    <t>Partial Trade Transfer</t>
   </si>
 </sst>
 </file>
@@ -561,13 +561,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -576,10 +576,10 @@
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -596,10 +596,10 @@
         <v>5</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="G2" s="2"/>
     </row>
@@ -617,13 +617,13 @@
         <v>5</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -640,10 +640,10 @@
         <v>7</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G4" s="2"/>
     </row>
@@ -661,14 +661,14 @@
         <v>7</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
@@ -685,13 +685,13 @@
         <v>5</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
@@ -705,13 +705,13 @@
         <v>21223</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G7" s="2"/>
     </row>
@@ -729,10 +729,10 @@
         <v>7</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="G8" s="2"/>
     </row>
@@ -750,13 +750,13 @@
         <v>7</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -773,10 +773,10 @@
         <v>7</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G10" s="2"/>
     </row>
@@ -791,17 +791,17 @@
         <v>23369</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -815,13 +815,13 @@
         <v>123456</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G12" s="2"/>
     </row>
@@ -836,17 +836,17 @@
         <v>123456</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="43.5" x14ac:dyDescent="0.35">
@@ -863,10 +863,10 @@
         <v>5</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G14" s="2"/>
     </row>

</xml_diff>

<commit_message>
More test data, UI changes, added snapshots
</commit_message>
<xml_diff>
--- a/ado-extract-partial-novation-phase1.xlsx
+++ b/ado-extract-partial-novation-phase1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chetan\ai-learning-lab\knowledge-drift-detector\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DFD818-12D0-49D4-9FF8-904D58F86077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D637EE-8362-489E-85A0-D66466C64676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{EB8649F9-5116-47FC-AF09-DC24D508B048}"/>
   </bookViews>
@@ -180,7 +180,7 @@
     <t>Partial Termination</t>
   </si>
   <si>
-    <t>Partial Trade Transfer</t>
+    <t>Partial Novation Phase 1</t>
   </si>
 </sst>
 </file>

</xml_diff>